<commit_message>
EPBDS-9967 Remove the ++ and -- operators, whose postfix value misleads users
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-9096-ConditionExpressionInvocationTest.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-9096-ConditionExpressionInvocationTest.xlsx
@@ -86,7 +86,7 @@
     <t>Steps</t>
   </si>
   <si>
-    <t>= indicator.times++</t>
+    <t>= indicator.times += 1</t>
   </si>
   <si>
     <t>Increment</t>
@@ -131,7 +131,7 @@
     <t>Spreadsheet Double doSomethingIntelligent2(Integer x, InvocationIndicator indicator)</t>
   </si>
   <si>
-    <t>= indicator.times2++</t>
+    <t>= indicator.times2 += 1</t>
   </si>
   <si>
     <t>= x-7</t>
@@ -140,7 +140,7 @@
     <t>Spreadsheet Double doSomethingIntelligent3(Integer x, InvocationIndicator indicator)</t>
   </si>
   <si>
-    <t>= indicator.times3++</t>
+    <t>= indicator.times3 += 1</t>
   </si>
   <si>
     <t>= x* 2</t>

</xml_diff>